<commit_message>
Order sheet: Kne Dag delivers daily, fish ordered Sunday for Monday
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PaCDQzCdGZVMUVUojbSF3f
</commit_message>
<xml_diff>
--- a/deliverables/max-savitz-orders-2026-10-19.xlsx
+++ b/deliverables/max-savitz-orders-2026-10-19.xlsx
@@ -53,7 +53,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F8D7D3"/>
+        <fgColor rgb="00DCEBE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -63,7 +63,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCEBE5"/>
+        <fgColor rgb="00F8D7D3"/>
       </patternFill>
     </fill>
   </fills>
@@ -563,10 +563,10 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="34" customHeight="1">
+    <row r="5" ht="22" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>קנה דג · דגים · להזמין: שישי 16/10 בבוקר — טלפון · אספקה: שני 19/10 בבוקר (אספקה מיוחדת!) · מספקים רק ג'/ה'/ו' — לסגור אספקה מיוחדת בשני, אחרת ספק אחר</t>
+          <t>קנה דג · דגים · להזמין: ראשון 18/10 · אספקה: שני 19/10 בבוקר</t>
         </is>
       </c>
     </row>
@@ -602,12 +602,12 @@
       <c r="G6" s="5" t="inlineStr"/>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>שישי 16/10 בבוקר — טלפון</t>
+          <t>ראשון 18/10</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>שני 19/10 בבוקר (אספקה מיוחדת!)</t>
+          <t>שני 19/10 בבוקר</t>
         </is>
       </c>
       <c r="J6" s="5" t="inlineStr">
@@ -652,12 +652,12 @@
       </c>
       <c r="H7" s="6" t="inlineStr">
         <is>
-          <t>שישי 16/10 בבוקר — טלפון</t>
+          <t>ראשון 18/10</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>שני 19/10 בבוקר (אספקה מיוחדת!)</t>
+          <t>שני 19/10 בבוקר</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -702,12 +702,12 @@
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>שישי 16/10 בבוקר — טלפון</t>
+          <t>ראשון 18/10</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>שני 19/10 בבוקר (אספקה מיוחדת!)</t>
+          <t>שני 19/10 בבוקר</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>גינדי בשר · בשר · להזמין: שבת/ראשון · אספקה: שני 19/10</t>
         </is>
@@ -866,7 +866,7 @@
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="7" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>משק הראל · ירקות · להזמין: ראשון 18/10 · אספקה: שני 19/10</t>
         </is>
@@ -2055,7 +2055,7 @@
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
-      <c r="A42" s="7" t="inlineStr">
+      <c r="A42" s="4" t="inlineStr">
         <is>
           <t>צ.י שיווק · חלבי · להזמין: ראשון 18/10 עד 18:00 · אספקה: שני 19/10</t>
         </is>
@@ -2442,7 +2442,7 @@
       </c>
     </row>
     <row r="52" ht="34" customHeight="1">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="7" t="inlineStr">
         <is>
           <t>דיפ שיווק · יבש · להזמין: עד שבת 17/10 13:00 · אספקה: ראשון 18/10 · לא מספקים בשני — אם מפספסים שבת 13:00 מגיע רק בשלישי</t>
         </is>
@@ -3109,7 +3109,7 @@
       </c>
     </row>
     <row r="68" ht="22" customHeight="1">
-      <c r="A68" s="7" t="inlineStr">
+      <c r="A68" s="4" t="inlineStr">
         <is>
           <t>לחמא · מאפים · להזמין: ראשון 18/10 עד 14:00 · אספקה: שני 19/10</t>
         </is>
@@ -3162,7 +3162,7 @@
       </c>
     </row>
     <row r="71" ht="22" customHeight="1">
-      <c r="A71" s="7" t="inlineStr">
+      <c r="A71" s="4" t="inlineStr">
         <is>
           <t>קנייה עצמית · מאפים · להזמין: שישי 16/10 · אספקה: —</t>
         </is>
@@ -3219,7 +3219,7 @@
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="7" t="inlineStr">
+      <c r="A74" s="4" t="inlineStr">
         <is>
           <t>דולצי · קינוחים · להזמין: ראשון 18/10 עד 10:00 · אספקה: שני 19/10</t>
         </is>
@@ -3276,7 +3276,7 @@
       </c>
     </row>
     <row r="77" ht="22" customHeight="1">
-      <c r="A77" s="7" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
         <is>
           <t>א. ביסקוטי · קינוחים · להזמין: לתאם · אספקה: לפני שני</t>
         </is>
@@ -3327,7 +3327,7 @@
       </c>
     </row>
     <row r="80" ht="22" customHeight="1">
-      <c r="A80" s="7" t="inlineStr">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>❓ לא ידוע · אחר · להזמין: לברר · אספקה: לברר</t>
         </is>
@@ -3490,17 +3490,17 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>שישי 16/10 בבוקר</t>
+          <t>שישי 16/10</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
-          <t>להתקשר לקנה דג — אספקה מיוחדת שני בבוקר (או ספק חלופי)</t>
+          <t>אריאל מאשר את כל השורות ⚠️ (אינטיאס, חמאה, ביצים/חלב, צנוברים, עשבים)</t>
         </is>
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t>ירין</t>
+          <t>אריאל</t>
         </is>
       </c>
     </row>
@@ -3512,12 +3512,12 @@
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>אריאל מאשר את כל השורות ⚠️ (אינטיאס, חמאה, ביצים/חלב, צנוברים, עשבים)</t>
+          <t>להזמין בשר לשני</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>אריאל</t>
+          <t>גינדי בשר</t>
         </is>
       </c>
     </row>
@@ -3529,63 +3529,63 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>להזמין בשר לשני</t>
+          <t>לקנות 6 חלות מתוקות</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>גינדי בשר</t>
+          <t>—</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>שישי 16/10</t>
+          <t>שבת 17/10 עד 13:00</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>לקנות 6 חלות מתוקות</t>
+          <t>הזמנת יבש (אספקה ראשון)</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>דיפ שיווק</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>שבת 17/10 עד 13:00</t>
+          <t>ראשון 18/10 בבוקר</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>הזמנת יבש (אספקה ראשון)</t>
+          <t>ספירת מלאי פסאו — להוריד מההזמנות מה שיש</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>דיפ שיווק</t>
+          <t>מטבח</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>ראשון 18/10 בבוקר</t>
+          <t>ראשון 18/10</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ספירת מלאי פסאו — להוריד מההזמנות מה שיש</t>
+          <t>דגים לשני בבוקר (טונה, אינטיאס, בר ים)</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>מטבח</t>
+          <t>קנה דג</t>
         </is>
       </c>
     </row>

</xml_diff>